<commit_message>
feat: integrate mech combat, commander UI and shared VFX updates
Include ground mech aim assist and flight changes, commander presentation and movement updates, and Excel-driven game text and VFX configuration.

Archive aim-assist build and import evidence; exclude the generated validation project copy. Editor build previously passed and Progress check has zero errors. No tests run in this session.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeMech.xlsx
+++ b/data/Excel/GuLiStrikeMech.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
   <si>
     <t>id</t>
   </si>
@@ -147,6 +147,126 @@
   </si>
   <si>
     <t>/Game/GuLiStrike/FX/GroundMech/NS_GroundMech_Muzzle.NS_GroundMech_Muzzle</t>
+  </si>
+  <si>
+    <t>ExecutionType</t>
+  </si>
+  <si>
+    <t>AbilityClass</t>
+  </si>
+  <si>
+    <t>MaxFuel</t>
+  </si>
+  <si>
+    <t>InitialFuel</t>
+  </si>
+  <si>
+    <t>FuelDrainPerSecond</t>
+  </si>
+  <si>
+    <t>FuelRecoveryPerSecond</t>
+  </si>
+  <si>
+    <t>FuelRecoveryDelay</t>
+  </si>
+  <si>
+    <t>ThrustAcceleration</t>
+  </si>
+  <si>
+    <t>MaxRiseSpeed</t>
+  </si>
+  <si>
+    <t>JetSystem</t>
+  </si>
+  <si>
+    <t>JetSocketLeft</t>
+  </si>
+  <si>
+    <t>JetSocketRight</t>
+  </si>
+  <si>
+    <t>JetScale</t>
+  </si>
+  <si>
+    <t>JetPitchDegrees</t>
+  </si>
+  <si>
+    <t>FuelBarMaterial</t>
+  </si>
+  <si>
+    <t>FuelBarHeight</t>
+  </si>
+  <si>
+    <t>FuelBarRightOffset</t>
+  </si>
+  <si>
+    <t>FuelBarFadeSeconds</t>
+  </si>
+  <si>
+    <t>Weapon</t>
+  </si>
+  <si>
+    <t>RocketJump</t>
+  </si>
+  <si>
+    <t>火箭跳；距离cm、时间s；空格持续推进，落地松键1秒后恢复；绿色1.5秒淡出</t>
+  </si>
+  <si>
+    <t>GAS</t>
+  </si>
+  <si>
+    <t>/Script/GuLiStrike.GuLiGA_RocketJump</t>
+  </si>
+  <si>
+    <t>/Game/Assets/VFX/WeaponBulletVFX/NS/VFX_FireGun_Loop.VFX_FireGun_Loop</t>
+  </si>
+  <si>
+    <t>Jet_Outlet_L</t>
+  </si>
+  <si>
+    <t>Jet_Outlet_R</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/GroundMech/UI/M_RocketFuelArc.M_RocketFuelArc</t>
+  </si>
+  <si>
+    <t>AirSpeedMultiplier</t>
+  </si>
+  <si>
+    <t>JetMaxTiltDegrees</t>
+  </si>
+  <si>
+    <t>火箭跳；距离cm、时间s；空格推进，落地松键1秒后恢复；未满常显，满后1.5秒淡出；空中WAD</t>
+  </si>
+  <si>
+    <t>火箭跳；距离cm、时间s；有效空格即时双喷并推进；落地松键1秒后恢复；未满常显，满后1.5秒淡出；空中WASD，下身随实际飞行方向，允许开火</t>
+  </si>
+  <si>
+    <t>FallGravityMultiplier</t>
+  </si>
+  <si>
+    <t>BulletVfxId</t>
+  </si>
+  <si>
+    <t>MuzzleVfxId</t>
+  </si>
+  <si>
+    <t>JetVfxId</t>
+  </si>
+  <si>
+    <t>FuelBarVfxId</t>
+  </si>
+  <si>
+    <t>AimAssistEnabled</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>AimAssistRadiusCentimeters</t>
+  </si>
+  <si>
+    <t>基础机枪；距离cm、时间s；射速/伤害只在升级表维护；辅助瞄准仅修正枪口，半径按目标深度投影</t>
   </si>
 </sst>
 </file>
@@ -626,6 +746,8 @@
     <col customWidth="true" max="2" min="1" width="23"/>
     <col customWidth="true" max="3" min="3" width="48"/>
     <col customWidth="true" max="14" min="4" width="23"/>
+    <col customWidth="true" max="34" min="15" width="25"/>
+    <col customWidth="true" max="36" min="35" width="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="true">
@@ -666,10 +788,76 @@
         <v>33</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>38</v>
+        <v>77</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="2">
@@ -710,10 +898,76 @@
         <v>34</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>31</v>
+        <v>14</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="AJ2" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -727,37 +981,103 @@
         <v>11</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>2</v>
+      <c r="P3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AH3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AI3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AJ3" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -768,7 +1088,7 @@
         <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>83</v>
       </c>
       <c r="D4">
         <v>12000</v>
@@ -797,11 +1117,103 @@
       <c r="L4" t="s">
         <v>35</v>
       </c>
-      <c r="M4" t="s">
-        <v>42</v>
-      </c>
-      <c r="N4" t="s">
-        <v>43</v>
+      <c r="M4">
+        <v>8</v>
+      </c>
+      <c r="N4">
+        <v>9</v>
+      </c>
+      <c r="O4" t="s">
+        <v>62</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AI4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AJ4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" t="s">
+        <v>74</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5" t="s">
+        <v>65</v>
+      </c>
+      <c r="P5" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q5">
+        <v>100</v>
+      </c>
+      <c r="R5">
+        <v>100</v>
+      </c>
+      <c r="S5">
+        <v>20</v>
+      </c>
+      <c r="T5">
+        <v>20</v>
+      </c>
+      <c r="U5">
+        <v>1</v>
+      </c>
+      <c r="V5">
+        <v>2180</v>
+      </c>
+      <c r="W5">
+        <v>1200</v>
+      </c>
+      <c r="X5">
+        <v>10</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>68</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>69</v>
+      </c>
+      <c r="AA5">
+        <v>-90</v>
+      </c>
+      <c r="AB5">
+        <v>11</v>
+      </c>
+      <c r="AC5">
+        <v>400</v>
+      </c>
+      <c r="AD5">
+        <v>450</v>
+      </c>
+      <c r="AE5">
+        <v>1.5</v>
+      </c>
+      <c r="AF5">
+        <v>1.5</v>
+      </c>
+      <c r="AG5">
+        <v>15</v>
+      </c>
+      <c r="AH5">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>